<commit_message>
fix duplicate weekends saturday and sunday
</commit_message>
<xml_diff>
--- a/output/DTR_7-4_rigor_Brando_Estanislao.xlsx
+++ b/output/DTR_7-4_rigor_Brando_Estanislao.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="66">
   <si>
     <t>Republic of the Philippines</t>
   </si>
@@ -68,6 +68,9 @@
     <t>Minutes</t>
   </si>
   <si>
+    <t>Sunday</t>
+  </si>
+  <si>
     <t>New Year</t>
   </si>
   <si>
@@ -77,9 +80,6 @@
     <t>Saturday</t>
   </si>
   <si>
-    <t>Sunday</t>
-  </si>
-  <si>
     <t>07:45</t>
   </si>
   <si>
@@ -101,130 +101,85 @@
     <t>16:01</t>
   </si>
   <si>
-    <t>07:07</t>
-  </si>
-  <si>
-    <t>11:00</t>
+    <t>07:32</t>
+  </si>
+  <si>
+    <t>16:09</t>
+  </si>
+  <si>
+    <t>07:27</t>
+  </si>
+  <si>
+    <t>11:44</t>
+  </si>
+  <si>
+    <t>17:01</t>
+  </si>
+  <si>
+    <t>06:40</t>
+  </si>
+  <si>
+    <t>11:01</t>
+  </si>
+  <si>
+    <t>11:31</t>
+  </si>
+  <si>
+    <t>16:02</t>
+  </si>
+  <si>
+    <t>06:51</t>
+  </si>
+  <si>
+    <t>11:03</t>
+  </si>
+  <si>
+    <t>11:40</t>
+  </si>
+  <si>
+    <t>07:29</t>
+  </si>
+  <si>
+    <t>11:15</t>
+  </si>
+  <si>
+    <t>11:34</t>
+  </si>
+  <si>
+    <t>07:04</t>
+  </si>
+  <si>
+    <t>11:21</t>
   </si>
   <si>
     <t>11:33</t>
   </si>
   <si>
-    <t>16:11</t>
-  </si>
-  <si>
-    <t>07:16</t>
-  </si>
-  <si>
-    <t>16:20</t>
-  </si>
-  <si>
-    <t>07:32</t>
-  </si>
-  <si>
-    <t>16:09</t>
-  </si>
-  <si>
-    <t>07:27</t>
-  </si>
-  <si>
-    <t>11:44</t>
-  </si>
-  <si>
-    <t>17:01</t>
-  </si>
-  <si>
-    <t>06:40</t>
-  </si>
-  <si>
-    <t>11:01</t>
-  </si>
-  <si>
-    <t>11:31</t>
-  </si>
-  <si>
-    <t>16:02</t>
-  </si>
-  <si>
-    <t>11:40</t>
-  </si>
-  <si>
-    <t>11:04</t>
-  </si>
-  <si>
-    <t>11:32</t>
-  </si>
-  <si>
-    <t>17:31</t>
-  </si>
-  <si>
-    <t>06:51</t>
-  </si>
-  <si>
-    <t>11:03</t>
-  </si>
-  <si>
-    <t>07:29</t>
-  </si>
-  <si>
-    <t>11:15</t>
-  </si>
-  <si>
-    <t>11:34</t>
-  </si>
-  <si>
-    <t>07:04</t>
-  </si>
-  <si>
-    <t>11:21</t>
-  </si>
-  <si>
     <t>17:12</t>
   </si>
   <si>
-    <t>06:56</t>
+    <t>07:25</t>
+  </si>
+  <si>
+    <t>11:07</t>
+  </si>
+  <si>
+    <t>11:39</t>
+  </si>
+  <si>
+    <t>16:10</t>
+  </si>
+  <si>
+    <t>07:31</t>
+  </si>
+  <si>
+    <t>11:38</t>
+  </si>
+  <si>
+    <t>06:49</t>
   </si>
   <si>
     <t>16:08</t>
-  </si>
-  <si>
-    <t>11:41</t>
-  </si>
-  <si>
-    <t>07:25</t>
-  </si>
-  <si>
-    <t>11:07</t>
-  </si>
-  <si>
-    <t>11:39</t>
-  </si>
-  <si>
-    <t>16:10</t>
-  </si>
-  <si>
-    <t>07:31</t>
-  </si>
-  <si>
-    <t>11:38</t>
-  </si>
-  <si>
-    <t>06:49</t>
-  </si>
-  <si>
-    <t>07:37</t>
-  </si>
-  <si>
-    <t>16:03</t>
-  </si>
-  <si>
-    <t>07:13</t>
-  </si>
-  <si>
-    <t>11:13</t>
-  </si>
-  <si>
-    <t>16:26</t>
   </si>
   <si>
     <t>11:02</t>
@@ -1172,10 +1127,12 @@
       <c r="C19" s="22"/>
       <c r="D19" s="22"/>
       <c r="E19" s="23"/>
-      <c r="F19" s="21"/>
+      <c r="F19" s="21" t="s">
+        <v>17</v>
+      </c>
       <c r="G19" s="21"/>
       <c r="H19" s="24" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I19" s="24"/>
       <c r="J19" s="24"/>
@@ -1191,7 +1148,7 @@
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
       <c r="H20" s="24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I20" s="24"/>
       <c r="J20" s="24"/>
@@ -1207,7 +1164,7 @@
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
       <c r="H21" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I21" s="25"/>
       <c r="J21" s="25"/>
@@ -1223,7 +1180,7 @@
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
       <c r="H22" s="25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I22" s="25"/>
       <c r="J22" s="25"/>
@@ -1276,19 +1233,13 @@
       <c r="A25" s="23">
         <v>7</v>
       </c>
-      <c r="B25" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="F25" s="21"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="21" t="s">
+        <v>20</v>
+      </c>
       <c r="G25" s="21"/>
       <c r="H25" s="25"/>
       <c r="I25" s="25"/>
@@ -1298,15 +1249,13 @@
       <c r="A26" s="23">
         <v>8</v>
       </c>
-      <c r="B26" s="22" t="s">
-        <v>32</v>
-      </c>
+      <c r="B26" s="22"/>
       <c r="C26" s="22"/>
       <c r="D26" s="22"/>
-      <c r="E26" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="F26" s="21"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="21" t="s">
+        <v>17</v>
+      </c>
       <c r="G26" s="21"/>
       <c r="H26" s="24"/>
       <c r="I26" s="24"/>
@@ -1317,12 +1266,12 @@
         <v>9</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C27" s="22"/>
       <c r="D27" s="22"/>
       <c r="E27" s="22" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F27" s="21"/>
       <c r="G27" s="21"/>
@@ -1341,7 +1290,7 @@
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
       <c r="H28" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I28" s="25"/>
       <c r="J28" s="25"/>
@@ -1357,7 +1306,7 @@
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
       <c r="H29" s="25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I29" s="25"/>
       <c r="J29" s="25"/>
@@ -1367,14 +1316,14 @@
         <v>12</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C30" s="22"/>
       <c r="D30" s="22" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
@@ -1387,16 +1336,16 @@
         <v>13</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="F31" s="21"/>
       <c r="G31" s="21"/>
@@ -1410,13 +1359,11 @@
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="22"/>
-      <c r="D32" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="E32" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="F32" s="21"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="21" t="s">
+        <v>20</v>
+      </c>
       <c r="G32" s="21"/>
       <c r="H32" s="25"/>
       <c r="I32" s="25"/>
@@ -1426,19 +1373,13 @@
       <c r="A33" s="23">
         <v>15</v>
       </c>
-      <c r="B33" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="F33" s="21"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="21" t="s">
+        <v>17</v>
+      </c>
       <c r="G33" s="21"/>
       <c r="H33" s="24"/>
       <c r="I33" s="24"/>
@@ -1449,13 +1390,13 @@
         <v>16</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>27</v>
@@ -1477,7 +1418,7 @@
       <c r="F35" s="21"/>
       <c r="G35" s="21"/>
       <c r="H35" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I35" s="25"/>
       <c r="J35" s="25"/>
@@ -1493,7 +1434,7 @@
       <c r="F36" s="21"/>
       <c r="G36" s="21"/>
       <c r="H36" s="25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I36" s="25"/>
       <c r="J36" s="25"/>
@@ -1503,16 +1444,16 @@
         <v>19</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F37" s="21"/>
       <c r="G37" s="21"/>
@@ -1525,16 +1466,16 @@
         <v>20</v>
       </c>
       <c r="B38" s="22" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F38" s="21"/>
       <c r="G38" s="21"/>
@@ -1546,19 +1487,13 @@
       <c r="A39" s="23">
         <v>21</v>
       </c>
-      <c r="B39" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D39" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="E39" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="F39" s="28"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="28" t="s">
+        <v>20</v>
+      </c>
       <c r="G39" s="28"/>
       <c r="H39" s="25"/>
       <c r="I39" s="25"/>
@@ -1569,16 +1504,12 @@
         <v>22</v>
       </c>
       <c r="B40" s="22"/>
-      <c r="C40" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="E40" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="F40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="21" t="s">
+        <v>17</v>
+      </c>
       <c r="G40" s="21"/>
       <c r="H40" s="25"/>
       <c r="I40" s="25"/>
@@ -1589,16 +1520,16 @@
         <v>23</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="F41" s="21"/>
       <c r="G41" s="21"/>
@@ -1617,7 +1548,7 @@
       <c r="F42" s="21"/>
       <c r="G42" s="21"/>
       <c r="H42" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I42" s="25"/>
       <c r="J42" s="25"/>
@@ -1633,7 +1564,7 @@
       <c r="F43" s="21"/>
       <c r="G43" s="21"/>
       <c r="H43" s="25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I43" s="25"/>
       <c r="J43" s="25"/>
@@ -1643,16 +1574,16 @@
         <v>26</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F44" s="21"/>
       <c r="G44" s="21"/>
@@ -1665,16 +1596,16 @@
         <v>27</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C45" s="22" t="s">
         <v>22</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F45" s="21"/>
       <c r="G45" s="21"/>
@@ -1686,19 +1617,13 @@
       <c r="A46" s="23">
         <v>28</v>
       </c>
-      <c r="B46" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D46" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="E46" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="F46" s="21"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="21" t="s">
+        <v>20</v>
+      </c>
       <c r="G46" s="21"/>
       <c r="H46" s="25"/>
       <c r="I46" s="25"/>
@@ -1708,19 +1633,13 @@
       <c r="A47" s="23">
         <v>29</v>
       </c>
-      <c r="B47" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="C47" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="D47" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E47" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="F47" s="21"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="21" t="s">
+        <v>17</v>
+      </c>
       <c r="G47" s="21"/>
       <c r="H47" s="25"/>
       <c r="I47" s="25"/>
@@ -1731,16 +1650,16 @@
         <v>30</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="F48" s="21"/>
       <c r="G48" s="21"/>
@@ -1759,14 +1678,14 @@
       <c r="F49" s="21"/>
       <c r="G49" s="21"/>
       <c r="H49" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I49" s="25"/>
       <c r="J49" s="25"/>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="29" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B50" s="29"/>
       <c r="C50" s="29"/>
@@ -1795,7 +1714,7 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="33" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="B52" s="13"/>
       <c r="C52" s="34"/>
@@ -1809,7 +1728,7 @@
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="13" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="B53" s="33"/>
       <c r="C53" s="34"/>
@@ -1850,7 +1769,7 @@
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="40" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="B56" s="40"/>
       <c r="C56" s="40"/>
@@ -1876,7 +1795,7 @@
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="42" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B58" s="43"/>
       <c r="C58" s="43"/>
@@ -1891,7 +1810,7 @@
     <row r="59" spans="1:10">
       <c r="A59" s="13"/>
       <c r="B59" s="45" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="C59" s="16"/>
       <c r="D59" s="16"/>
@@ -1916,7 +1835,7 @@
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="47" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="B61" s="47"/>
       <c r="C61" s="47"/>
@@ -1930,7 +1849,7 @@
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="16" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="16"/>

</xml_diff>